<commit_message>
[feat] update optimization programs for 3 objects
</commit_message>
<xml_diff>
--- a/simulation/torque_AG.xlsx
+++ b/simulation/torque_AG.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ou918\ECB_project\simulation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0CA6080-D5BD-4176-9487-98CC1CF287D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAAC5FCB-C575-4347-8A14-B8F183C47DC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{39CA443E-9F7F-4F8D-96E7-717943A268F3}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{39CA443E-9F7F-4F8D-96E7-717943A268F3}"/>
   </bookViews>
   <sheets>
     <sheet name="AGmax_4" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="9">
   <si>
     <t>AG [mm]</t>
   </si>
@@ -66,6 +66,10 @@
   </si>
   <si>
     <t>error</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Kenny</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -237,7 +241,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -415,6 +419,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -665,7 +675,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -682,6 +692,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="14" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="33" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -6977,14 +6993,14 @@
       <c r="D151">
         <v>1.7991066069999999</v>
       </c>
-      <c r="E151">
+      <c r="E151" s="6">
         <f>AVERAGE(D151:D156)</f>
         <v>1.8028853129999998</v>
       </c>
-      <c r="F151">
+      <c r="F151" s="6">
         <v>1.833</v>
       </c>
-      <c r="G151" s="1">
+      <c r="G151" s="7">
         <f>(E151-F151)/F151</f>
         <v>-1.6429180032733331E-2</v>
       </c>
@@ -10104,7 +10120,7 @@
         <v>-0.12188761887488714</v>
       </c>
     </row>
-    <row r="369" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A369">
         <v>0</v>
       </c>
@@ -10118,7 +10134,7 @@
         <v>3.5490030720000001</v>
       </c>
     </row>
-    <row r="370" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A370">
         <v>0</v>
       </c>
@@ -10132,7 +10148,7 @@
         <v>3.5571972600000001</v>
       </c>
     </row>
-    <row r="371" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A371">
         <v>0</v>
       </c>
@@ -10146,7 +10162,7 @@
         <v>3.5649804340000002</v>
       </c>
     </row>
-    <row r="372" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A372">
         <v>0</v>
       </c>
@@ -10160,7 +10176,7 @@
         <v>3.5853881429999999</v>
       </c>
     </row>
-    <row r="373" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A373">
         <v>0</v>
       </c>
@@ -10174,7 +10190,25 @@
         <v>3.5910562869999998</v>
       </c>
     </row>
-    <row r="381" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G374" s="1"/>
+    </row>
+    <row r="375" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D375" t="s">
+        <v>8</v>
+      </c>
+      <c r="E375">
+        <v>1.81</v>
+      </c>
+      <c r="F375">
+        <v>1.701716</v>
+      </c>
+      <c r="G375" s="1">
+        <f>(E375-F375)/F375</f>
+        <v>6.363223945711273E-2</v>
+      </c>
+    </row>
+    <row r="381" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
         <v>0</v>
       </c>
@@ -10191,7 +10225,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="382" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A382">
         <v>0</v>
       </c>
@@ -10212,7 +10246,7 @@
         <v>3.8618508474908032E-2</v>
       </c>
     </row>
-    <row r="383" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A383">
         <v>0</v>
       </c>
@@ -10233,7 +10267,7 @@
         <v>1.392744813002977E-2</v>
       </c>
     </row>
-    <row r="384" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A384">
         <v>0</v>
       </c>
@@ -10466,7 +10500,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B2B8C80-D88D-405B-B7D1-788DDAEC3F43}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:F357"/>
+  <dimension ref="A1:F358"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="10.625" bestFit="1" customWidth="1"/>
@@ -15332,7 +15366,7 @@
         <v>3.3888328719402798</v>
       </c>
       <c r="E345" s="1">
-        <f t="shared" ref="E345:E356" si="0">(C345-D345)/D345</f>
+        <f t="shared" ref="E345:E358" si="0">(C345-D345)/D345</f>
         <v>0.11302763976094669</v>
       </c>
       <c r="F345">
@@ -15574,9 +15608,25 @@
       </c>
     </row>
     <row r="357" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E357" s="5"/>
       <c r="F357" s="1">
         <f>AVERAGE(F345:F356)</f>
         <v>7.3782001474630696E-2</v>
+      </c>
+    </row>
+    <row r="358" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B358" t="s">
+        <v>8</v>
+      </c>
+      <c r="C358">
+        <v>18.177</v>
+      </c>
+      <c r="D358">
+        <v>18.13</v>
+      </c>
+      <c r="E358" s="5">
+        <f t="shared" si="0"/>
+        <v>2.5923883066740539E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>